<commit_message>
Update A-Share Blast Lab / 2026-10-25 theme-integration-manual
</commit_message>
<xml_diff>
--- a/data/five_break_10_targets.xlsx
+++ b/data/five_break_10_targets.xlsx
@@ -7979,34 +7979,34 @@
         <v>20.45</v>
       </c>
       <c r="H115" s="3" t="n">
-        <v>23.96</v>
+        <v>24.01</v>
       </c>
       <c r="I115" s="4" t="n">
-        <v>17.16381418092909</v>
+        <v>17.40831295843521</v>
       </c>
       <c r="J115" s="3" t="n">
         <v>24.54</v>
       </c>
       <c r="K115" s="3" t="n">
-        <v>21.31</v>
+        <v>21.32</v>
       </c>
       <c r="L115" s="3" t="n">
-        <v>21.711</v>
+        <v>21.731</v>
       </c>
       <c r="M115" s="4" t="n">
-        <v>-1.84699000506654</v>
+        <v>-1.891307348948501</v>
       </c>
       <c r="N115" s="3" t="n">
-        <v>21.902</v>
+        <v>21.922</v>
       </c>
       <c r="O115" s="3" t="n">
-        <v>21.901</v>
+        <v>21.921</v>
       </c>
       <c r="P115" s="4" t="n">
-        <v>0.004566001552452903</v>
+        <v>0.004561835682692639</v>
       </c>
       <c r="Q115" s="5" t="n">
-        <v>1.851556006618993</v>
+        <v>1.895869184631194</v>
       </c>
       <c r="R115" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update A-Share Blast Lab / 2026-10-26 remove-reversal-and-groups
</commit_message>
<xml_diff>
--- a/data/five_break_10_targets.xlsx
+++ b/data/five_break_10_targets.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="监控结果" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'监控结果'!$A$2:$R$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'监控结果'!$A$2:$R$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R77"/>
+  <dimension ref="A1:R76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -471,7 +471,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>5破10明日门槛完整名单｜信号日 2026-10-26｜75 只｜报告 多空阶段_2026-10-26.xlsx</t>
+          <t>5破10明日门槛完整名单｜信号日 2026-10-26｜74 只｜报告 多空阶段_2026-10-26.xlsx</t>
         </is>
       </c>
     </row>
@@ -5425,76 +5425,8 @@
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>商业航天</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>空转多</t>
-        </is>
-      </c>
-      <c r="D77" t="n">
-        <v>1</v>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>002115</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>三维通信</t>
-        </is>
-      </c>
-      <c r="G77" s="3" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="H77" s="3" t="n">
-        <v>10.63</v>
-      </c>
-      <c r="I77" s="4" t="n">
-        <v>9.587628865979392</v>
-      </c>
-      <c r="J77" s="3" t="n">
-        <v>10.67</v>
-      </c>
-      <c r="K77" s="3" t="n">
-        <v>9.746</v>
-      </c>
-      <c r="L77" s="3" t="n">
-        <v>9.763</v>
-      </c>
-      <c r="M77" s="4" t="n">
-        <v>-0.1741268052852574</v>
-      </c>
-      <c r="N77" s="3" t="n">
-        <v>9.918000000000001</v>
-      </c>
-      <c r="O77" s="3" t="n">
-        <v>9.788</v>
-      </c>
-      <c r="P77" s="4" t="n">
-        <v>1.328156926849222</v>
-      </c>
-      <c r="Q77" s="5" t="n">
-        <v>1.50228373213448</v>
-      </c>
-      <c r="R77" t="inlineStr">
-        <is>
-          <t>涨停内可达</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:R77"/>
+  <autoFilter ref="A2:R76"/>
   <mergeCells count="1">
     <mergeCell ref="A1:R1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Update A-Share Blast Lab / 2026-10-27 monitor-schedule-0915-1501
</commit_message>
<xml_diff>
--- a/data/five_break_10_targets.xlsx
+++ b/data/five_break_10_targets.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="监控结果" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'监控结果'!$A$2:$R$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'监控结果'!$A$2:$R$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R76"/>
+  <dimension ref="A1:R77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -471,7 +471,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>5破10明日门槛完整名单｜信号日 2026-10-26｜74 只｜报告 多空阶段_2026-10-26.xlsx</t>
+          <t>5破10明日门槛完整名单｜信号日 2026-10-26｜75 只｜报告 多空阶段_2026-10-26.xlsx</t>
         </is>
       </c>
     </row>
@@ -5425,8 +5425,76 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>商业航天</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>空转多</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>002115</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>三维通信</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="H77" s="3" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="I77" s="4" t="n">
+        <v>9.587628865979392</v>
+      </c>
+      <c r="J77" s="3" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="K77" s="3" t="n">
+        <v>9.746</v>
+      </c>
+      <c r="L77" s="3" t="n">
+        <v>9.763</v>
+      </c>
+      <c r="M77" s="4" t="n">
+        <v>-0.1741268052852574</v>
+      </c>
+      <c r="N77" s="3" t="n">
+        <v>9.918000000000001</v>
+      </c>
+      <c r="O77" s="3" t="n">
+        <v>9.788</v>
+      </c>
+      <c r="P77" s="4" t="n">
+        <v>1.328156926849222</v>
+      </c>
+      <c r="Q77" s="5" t="n">
+        <v>1.50228373213448</v>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>涨停内可达</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:R76"/>
+  <autoFilter ref="A2:R77"/>
   <mergeCells count="1">
     <mergeCell ref="A1:R1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Update A-Share Blast Lab / 2026-10-28 09:30
</commit_message>
<xml_diff>
--- a/data/five_break_10_targets.xlsx
+++ b/data/five_break_10_targets.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="监控结果" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'监控结果'!$A$2:$R$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'监控结果'!$A$2:$R$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R90"/>
+  <dimension ref="A1:R92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -471,7 +471,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>5破10明日门槛完整名单｜信号日 2026-10-27｜88 只｜报告 多空阶段_2026-10-27.xlsx</t>
+          <t>5破10明日门槛完整名单｜信号日 2026-10-27｜90 只｜报告 多空阶段_2026-10-27.xlsx</t>
         </is>
       </c>
     </row>
@@ -2330,7 +2330,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>互金证券</t>
+          <t>AI应用</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2343,46 +2343,46 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>600621</t>
+          <t>301052</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>华鑫股份</t>
+          <t>果麦文化</t>
         </is>
       </c>
       <c r="G30" s="3" t="n">
-        <v>14.9</v>
+        <v>32.45</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>15.91</v>
+        <v>34.69</v>
       </c>
       <c r="I30" s="4" t="n">
-        <v>6.778523489932886</v>
+        <v>6.902927580893659</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>16.39</v>
+        <v>38.94</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>14.66</v>
+        <v>32.11799999999999</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>14.77</v>
+        <v>33.262</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>-0.7447528774542911</v>
+        <v>-3.439360230894128</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>14.996</v>
+        <v>33.19600000000001</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>14.883</v>
+        <v>33.194</v>
       </c>
       <c r="P30" s="4" t="n">
-        <v>0.7592555264395617</v>
+        <v>0.006025185274460831</v>
       </c>
       <c r="Q30" s="5" t="n">
-        <v>1.504008403893853</v>
+        <v>3.445385416168589</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
@@ -2398,56 +2398,59 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>互金证券</t>
+          <t>AI应用</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>空</t>
-        </is>
+          <t>空转多</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>3</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>601519</t>
+          <t>603258</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>大智慧</t>
+          <t>电魂网络</t>
         </is>
       </c>
       <c r="G31" s="3" t="n">
-        <v>8.76</v>
+        <v>15</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>9.390000000000001</v>
+        <v>16.16</v>
       </c>
       <c r="I31" s="4" t="n">
-        <v>7.191780821917826</v>
+        <v>7.733333333333325</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>9.630000000000001</v>
+        <v>16.5</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>9.022</v>
+        <v>14.786</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>9.144000000000002</v>
+        <v>14.95</v>
       </c>
       <c r="M31" s="4" t="n">
-        <v>-1.334208223972022</v>
+        <v>-1.096989966555195</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>9.218</v>
+        <v>15.306</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>9.118</v>
+        <v>14.885</v>
       </c>
       <c r="P31" s="4" t="n">
-        <v>1.096731739416534</v>
+        <v>2.828350688612713</v>
       </c>
       <c r="Q31" s="5" t="n">
-        <v>2.430939963388556</v>
+        <v>3.925340655167908</v>
       </c>
       <c r="R31" t="inlineStr">
         <is>
@@ -2463,7 +2466,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>互金证券</t>
+          <t>AI应用</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2473,46 +2476,46 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>600958</t>
+          <t>300251</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>东方证券</t>
+          <t>光线传媒</t>
         </is>
       </c>
       <c r="G32" s="3" t="n">
-        <v>8.48</v>
+        <v>11.59</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>9.15</v>
+        <v>12.01</v>
       </c>
       <c r="I32" s="4" t="n">
-        <v>7.900943396226423</v>
+        <v>3.623813632441752</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>9.32</v>
+        <v>13.9</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>8.586</v>
+        <v>11.622</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>8.595000000000002</v>
+        <v>11.649</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>-0.1047120418848468</v>
+        <v>-0.2317795518928856</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>8.75</v>
+        <v>11.816</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>8.629</v>
+        <v>11.668</v>
       </c>
       <c r="P32" s="4" t="n">
-        <v>1.402248232703673</v>
+        <v>1.26842646554679</v>
       </c>
       <c r="Q32" s="5" t="n">
-        <v>1.50696027458852</v>
+        <v>1.500206017439676</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
@@ -2528,7 +2531,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>互金证券</t>
+          <t>AI应用</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2538,46 +2541,46 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>601377</t>
+          <t>300133</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>兴业证券</t>
+          <t>华策影视</t>
         </is>
       </c>
       <c r="G33" s="3" t="n">
-        <v>5.52</v>
+        <v>8.92</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>6</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="I33" s="4" t="n">
-        <v>8.695652173913061</v>
+        <v>5.94170403587444</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>6.07</v>
+        <v>10.7</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>5.613999999999999</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>5.625999999999999</v>
+        <v>9.052000000000001</v>
       </c>
       <c r="M33" s="4" t="n">
-        <v>-0.2132954141486065</v>
+        <v>-1.789659743703054</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>5.726</v>
+        <v>9.059999999999999</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>5.653</v>
+        <v>9.058000000000002</v>
       </c>
       <c r="P33" s="4" t="n">
-        <v>1.291349725809288</v>
+        <v>0.02207992934419867</v>
       </c>
       <c r="Q33" s="5" t="n">
-        <v>1.504645139957894</v>
+        <v>1.811739673047252</v>
       </c>
       <c r="R33" t="inlineStr">
         <is>
@@ -2593,7 +2596,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>互金证券</t>
+          <t>AI应用</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2603,46 +2606,46 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>002736</t>
+          <t>002400</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>国信证券</t>
+          <t>省广集团</t>
         </is>
       </c>
       <c r="G34" s="3" t="n">
-        <v>9.66</v>
+        <v>6.45</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>10.52</v>
+        <v>6.85</v>
       </c>
       <c r="I34" s="4" t="n">
-        <v>8.902691511387161</v>
+        <v>6.201550387596888</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>10.62</v>
+        <v>7.09</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>9.806000000000001</v>
+        <v>6.525999999999999</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>9.812999999999999</v>
+        <v>6.565</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>-0.07133394476712684</v>
+        <v>-0.5940594059406057</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>10.008</v>
+        <v>6.641999999999999</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>9.866999999999999</v>
+        <v>6.581999999999999</v>
       </c>
       <c r="P34" s="4" t="n">
-        <v>1.429005776831871</v>
+        <v>0.9115770282588809</v>
       </c>
       <c r="Q34" s="5" t="n">
-        <v>1.500339721598998</v>
+        <v>1.505636434199487</v>
       </c>
       <c r="R34" t="inlineStr">
         <is>
@@ -2658,7 +2661,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>互金证券</t>
+          <t>AI应用</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2668,46 +2671,46 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>601136</t>
+          <t>002555</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>首创证券</t>
+          <t>三七互娱</t>
         </is>
       </c>
       <c r="G35" s="3" t="n">
-        <v>13.49</v>
+        <v>16.1</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>14.78</v>
+        <v>17.29</v>
       </c>
       <c r="I35" s="4" t="n">
-        <v>9.562638991845795</v>
+        <v>7.391304347826066</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>14.83</v>
+        <v>17.71</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>13.94</v>
+        <v>16.418</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>14.029</v>
+        <v>16.676</v>
       </c>
       <c r="M35" s="4" t="n">
-        <v>-0.6344001710741898</v>
+        <v>-1.547133605181095</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>14.184</v>
+        <v>16.684</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>14.062</v>
+        <v>16.678</v>
       </c>
       <c r="P35" s="4" t="n">
-        <v>0.8675864030721181</v>
+        <v>0.03597553663508002</v>
       </c>
       <c r="Q35" s="5" t="n">
-        <v>1.501986574146308</v>
+        <v>1.583109141816175</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
@@ -2723,7 +2726,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>互金证券</t>
+          <t>AI应用</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2733,46 +2736,46 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>688318</t>
+          <t>300418</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>财富趋势</t>
+          <t>昆仑万维</t>
         </is>
       </c>
       <c r="G36" s="3" t="n">
-        <v>69.98999999999999</v>
+        <v>39.19</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>77.61</v>
+        <v>42.11</v>
       </c>
       <c r="I36" s="4" t="n">
-        <v>10.88726960994428</v>
+        <v>7.45088032661394</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>83.98</v>
+        <v>47.02</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>73.66400000000002</v>
+        <v>39.884</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>73.70700000000001</v>
+        <v>40.01</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>-0.05833909940710091</v>
+        <v>-0.3149212696825776</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>75.06800000000001</v>
+        <v>40.746</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>74.001</v>
+        <v>40.009</v>
       </c>
       <c r="P36" s="4" t="n">
-        <v>1.441872407129652</v>
+        <v>1.842085530755577</v>
       </c>
       <c r="Q36" s="5" t="n">
-        <v>1.500211506536753</v>
+        <v>2.157006800438155</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
@@ -2788,7 +2791,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>互金证券</t>
+          <t>AI应用</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2798,46 +2801,46 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>300803</t>
+          <t>600986</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>指南针</t>
+          <t>浙文互联</t>
         </is>
       </c>
       <c r="G37" s="3" t="n">
-        <v>48.38</v>
+        <v>6.79</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>55.17</v>
+        <v>7.34</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>14.03472509301364</v>
+        <v>8.100147275405</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>58.05</v>
+        <v>7.46</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>51.812</v>
+        <v>6.907999999999999</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>52.057</v>
+        <v>6.93</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>-0.4706379545498129</v>
+        <v>-0.3174603174603163</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>52.79600000000001</v>
+        <v>7.058</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>52.258</v>
+        <v>6.953999999999999</v>
       </c>
       <c r="P37" s="4" t="n">
-        <v>1.029507443836364</v>
+        <v>1.495542134023609</v>
       </c>
       <c r="Q37" s="5" t="n">
-        <v>1.500145398386177</v>
+        <v>1.813002451483925</v>
       </c>
       <c r="R37" t="inlineStr">
         <is>
@@ -2853,7 +2856,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>互金证券</t>
+          <t>AI应用</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2863,46 +2866,46 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>300085</t>
+          <t>600556</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>银之杰</t>
+          <t>天下秀</t>
         </is>
       </c>
       <c r="G38" s="3" t="n">
-        <v>24.89</v>
+        <v>4.68</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>28.83</v>
+        <v>5.06</v>
       </c>
       <c r="I38" s="4" t="n">
-        <v>15.82965046203293</v>
+        <v>8.119658119658112</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>29.86</v>
+        <v>5.14</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>26.71</v>
+        <v>4.81</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>26.998</v>
+        <v>4.857</v>
       </c>
       <c r="M38" s="4" t="n">
-        <v>-1.066745684865533</v>
+        <v>-0.9676755198682274</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>27.322</v>
+        <v>4.895999999999999</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>27.123</v>
+        <v>4.867</v>
       </c>
       <c r="P38" s="4" t="n">
-        <v>0.7336946502968011</v>
+        <v>0.5958495993424906</v>
       </c>
       <c r="Q38" s="5" t="n">
-        <v>1.800440335162334</v>
+        <v>1.563525119210718</v>
       </c>
       <c r="R38" t="inlineStr">
         <is>
@@ -2923,54 +2926,51 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>空转多</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>3</v>
+          <t>空</t>
+        </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>301052</t>
+          <t>603444</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>果麦文化</t>
+          <t>吉比特</t>
         </is>
       </c>
       <c r="G39" s="3" t="n">
-        <v>32.45</v>
+        <v>328.69</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>34.69</v>
+        <v>358.12</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>6.902927580893659</v>
+        <v>8.953725394748858</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>38.94</v>
+        <v>361.55</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>32.11799999999999</v>
+        <v>332.52</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>33.262</v>
+        <v>334.83</v>
       </c>
       <c r="M39" s="4" t="n">
-        <v>-3.439360230894128</v>
+        <v>-0.6899023385001368</v>
       </c>
       <c r="N39" s="3" t="n">
-        <v>33.19600000000001</v>
+        <v>339.542</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>33.194</v>
+        <v>336.813</v>
       </c>
       <c r="P39" s="4" t="n">
-        <v>0.006025185274460831</v>
+        <v>0.8102418849628812</v>
       </c>
       <c r="Q39" s="5" t="n">
-        <v>3.445385416168589</v>
+        <v>1.500144223463018</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
@@ -2991,54 +2991,51 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>空转多</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>3</v>
+          <t>空</t>
+        </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>603258</t>
+          <t>300182</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>电魂网络</t>
+          <t>捷成股份</t>
         </is>
       </c>
       <c r="G40" s="3" t="n">
-        <v>15</v>
+        <v>5.33</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>16.16</v>
+        <v>5.9</v>
       </c>
       <c r="I40" s="4" t="n">
-        <v>7.733333333333325</v>
+        <v>10.69418386491559</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>16.5</v>
+        <v>6.39</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>14.786</v>
+        <v>5.526000000000001</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>14.95</v>
+        <v>5.555000000000001</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>-1.096989966555195</v>
+        <v>-0.5220522052205245</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>15.306</v>
+        <v>5.648</v>
       </c>
       <c r="O40" s="3" t="n">
-        <v>14.885</v>
+        <v>5.58</v>
       </c>
       <c r="P40" s="4" t="n">
-        <v>2.828350688612713</v>
+        <v>1.218637992831528</v>
       </c>
       <c r="Q40" s="5" t="n">
-        <v>3.925340655167908</v>
+        <v>1.740690198052053</v>
       </c>
       <c r="R40" t="inlineStr">
         <is>
@@ -3064,46 +3061,46 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>300251</t>
+          <t>300364</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>光线传媒</t>
+          <t>中文在线</t>
         </is>
       </c>
       <c r="G41" s="3" t="n">
-        <v>11.59</v>
+        <v>23.45</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>12.01</v>
+        <v>26.59</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>3.623813632441752</v>
+        <v>13.39019189765458</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>13.9</v>
+        <v>28.14</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>11.622</v>
+        <v>24.172</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>11.649</v>
+        <v>24.289</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>-0.2317795518928856</v>
+        <v>-0.4816995347688091</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>11.816</v>
+        <v>24.904</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>11.668</v>
+        <v>24.422</v>
       </c>
       <c r="P41" s="4" t="n">
-        <v>1.26842646554679</v>
+        <v>1.973630333306042</v>
       </c>
       <c r="Q41" s="5" t="n">
-        <v>1.500206017439676</v>
+        <v>2.455329868074851</v>
       </c>
       <c r="R41" t="inlineStr">
         <is>
@@ -3129,46 +3126,46 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>300133</t>
+          <t>300063</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>华策影视</t>
+          <t>天龙集团</t>
         </is>
       </c>
       <c r="G42" s="3" t="n">
-        <v>8.92</v>
+        <v>7.93</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>9.449999999999999</v>
+        <v>9.01</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>5.94170403587444</v>
+        <v>13.61916771752838</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>10.7</v>
+        <v>9.51</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>8.890000000000001</v>
+        <v>8.251999999999999</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>9.052000000000001</v>
+        <v>8.348000000000001</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>-1.789659743703054</v>
+        <v>-1.149976042165812</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>9.059999999999999</v>
+        <v>8.484</v>
       </c>
       <c r="O42" s="3" t="n">
-        <v>9.058000000000002</v>
+        <v>8.375</v>
       </c>
       <c r="P42" s="4" t="n">
-        <v>0.02207992934419867</v>
+        <v>1.301492537313442</v>
       </c>
       <c r="Q42" s="5" t="n">
-        <v>1.811739673047252</v>
+        <v>2.451468579479255</v>
       </c>
       <c r="R42" t="inlineStr">
         <is>
@@ -3194,46 +3191,46 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>002400</t>
+          <t>301262</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>省广集团</t>
+          <t>海看股份</t>
         </is>
       </c>
       <c r="G43" s="3" t="n">
-        <v>6.45</v>
+        <v>20.35</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>6.85</v>
+        <v>23.42</v>
       </c>
       <c r="I43" s="4" t="n">
-        <v>6.201550387596888</v>
+        <v>15.08599508599509</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>7.09</v>
+        <v>24.42</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>6.525999999999999</v>
+        <v>20.926</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>6.565</v>
+        <v>21.222</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>-0.5940594059406057</v>
+        <v>-1.394779002921476</v>
       </c>
       <c r="N43" s="3" t="n">
-        <v>6.641999999999999</v>
+        <v>21.662</v>
       </c>
       <c r="O43" s="3" t="n">
-        <v>6.581999999999999</v>
+        <v>21.348</v>
       </c>
       <c r="P43" s="4" t="n">
-        <v>0.9115770282588809</v>
+        <v>1.470863781150444</v>
       </c>
       <c r="Q43" s="5" t="n">
-        <v>1.505636434199487</v>
+        <v>2.86564278407192</v>
       </c>
       <c r="R43" t="inlineStr">
         <is>
@@ -3259,46 +3256,46 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>002555</t>
+          <t>300959</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>三七互娱</t>
+          <t>线上线下</t>
         </is>
       </c>
       <c r="G44" s="3" t="n">
-        <v>16.1</v>
+        <v>68.5</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>17.29</v>
+        <v>79.03</v>
       </c>
       <c r="I44" s="4" t="n">
-        <v>7.391304347826066</v>
+        <v>15.37226277372263</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>17.71</v>
+        <v>82.2</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>16.418</v>
+        <v>72.27799999999999</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>16.676</v>
+        <v>73.40299999999999</v>
       </c>
       <c r="M44" s="4" t="n">
-        <v>-1.547133605181095</v>
+        <v>-1.532634905930275</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>16.684</v>
+        <v>74.042</v>
       </c>
       <c r="O44" s="3" t="n">
-        <v>16.678</v>
+        <v>73.756</v>
       </c>
       <c r="P44" s="4" t="n">
-        <v>0.03597553663508002</v>
+        <v>0.3877650631813001</v>
       </c>
       <c r="Q44" s="5" t="n">
-        <v>1.583109141816175</v>
+        <v>1.920399969111575</v>
       </c>
       <c r="R44" t="inlineStr">
         <is>
@@ -3324,46 +3321,46 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>300418</t>
+          <t>300785</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>昆仑万维</t>
+          <t>值得买</t>
         </is>
       </c>
       <c r="G45" s="3" t="n">
-        <v>39.19</v>
+        <v>32.47</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>42.11</v>
+        <v>37.95</v>
       </c>
       <c r="I45" s="4" t="n">
-        <v>7.45088032661394</v>
+        <v>16.87711733908224</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>47.02</v>
+        <v>38.96</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>39.884</v>
+        <v>34.376</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>40.01</v>
+        <v>34.82600000000001</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>-0.3149212696825776</v>
+        <v>-1.292138057772951</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>40.746</v>
+        <v>35.33</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>40.009</v>
+        <v>35.05500000000001</v>
       </c>
       <c r="P45" s="4" t="n">
-        <v>1.842085530755577</v>
+        <v>0.7844815290257934</v>
       </c>
       <c r="Q45" s="5" t="n">
-        <v>2.157006800438155</v>
+        <v>2.076619586798745</v>
       </c>
       <c r="R45" t="inlineStr">
         <is>
@@ -3389,46 +3386,46 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>600986</t>
+          <t>301171</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>浙文互联</t>
+          <t>易点天下</t>
         </is>
       </c>
       <c r="G46" s="3" t="n">
-        <v>6.79</v>
+        <v>28.9</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>7.34</v>
+        <v>33.87</v>
       </c>
       <c r="I46" s="4" t="n">
-        <v>8.100147275405</v>
+        <v>17.19723183391002</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>7.46</v>
+        <v>34.68</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>6.907999999999999</v>
+        <v>30.872</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>6.93</v>
+        <v>30.89</v>
       </c>
       <c r="M46" s="4" t="n">
-        <v>-0.3174603174603163</v>
+        <v>-0.0582712852055467</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>7.058</v>
+        <v>31.734</v>
       </c>
       <c r="O46" s="3" t="n">
-        <v>6.953999999999999</v>
+        <v>31.077</v>
       </c>
       <c r="P46" s="4" t="n">
-        <v>1.495542134023609</v>
+        <v>2.11410367796121</v>
       </c>
       <c r="Q46" s="5" t="n">
-        <v>1.813002451483925</v>
+        <v>2.172374963166757</v>
       </c>
       <c r="R46" t="inlineStr">
         <is>
@@ -3444,7 +3441,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>AI应用</t>
+          <t>机器人</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3454,46 +3451,46 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>600556</t>
+          <t>301182</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>天下秀</t>
+          <t>凯旺科技</t>
         </is>
       </c>
       <c r="G47" s="3" t="n">
-        <v>4.68</v>
+        <v>43.21</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>5.06</v>
+        <v>50.56</v>
       </c>
       <c r="I47" s="4" t="n">
-        <v>8.119658119658112</v>
+        <v>17.00995140013886</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>5.14</v>
+        <v>51.85</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>4.81</v>
+        <v>46.172</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>4.857</v>
+        <v>46.638</v>
       </c>
       <c r="M47" s="4" t="n">
-        <v>-0.9676755198682274</v>
+        <v>-0.9991852137741675</v>
       </c>
       <c r="N47" s="3" t="n">
-        <v>4.895999999999999</v>
+        <v>47.264</v>
       </c>
       <c r="O47" s="3" t="n">
-        <v>4.867</v>
+        <v>46.95</v>
       </c>
       <c r="P47" s="4" t="n">
-        <v>0.5958495993424906</v>
+        <v>0.6687965921192696</v>
       </c>
       <c r="Q47" s="5" t="n">
-        <v>1.563525119210718</v>
+        <v>1.667981805893437</v>
       </c>
       <c r="R47" t="inlineStr">
         <is>
@@ -3509,7 +3506,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>AI应用</t>
+          <t>机器人</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3519,46 +3516,46 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>603444</t>
+          <t>688697</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>吉比特</t>
+          <t>纽威数控</t>
         </is>
       </c>
       <c r="G48" s="3" t="n">
-        <v>328.69</v>
+        <v>11.76</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>358.12</v>
+        <v>13.78</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>8.953725394748858</v>
+        <v>17.17687074829932</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>361.55</v>
+        <v>14.11</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>332.52</v>
+        <v>12.474</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>334.83</v>
+        <v>12.548</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>-0.6899023385001368</v>
+        <v>-0.5897354160025459</v>
       </c>
       <c r="N48" s="3" t="n">
-        <v>339.542</v>
+        <v>12.832</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>336.813</v>
+        <v>12.656</v>
       </c>
       <c r="P48" s="4" t="n">
-        <v>0.8102418849628812</v>
+        <v>1.390644753476589</v>
       </c>
       <c r="Q48" s="5" t="n">
-        <v>1.500144223463018</v>
+        <v>1.980380169479135</v>
       </c>
       <c r="R48" t="inlineStr">
         <is>
@@ -3574,56 +3571,59 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>AI应用</t>
+          <t>药</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>空</t>
-        </is>
+          <t>空转多</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>300182</t>
+          <t>600380</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>捷成股份</t>
+          <t>健康元</t>
         </is>
       </c>
       <c r="G49" s="3" t="n">
-        <v>5.33</v>
+        <v>9.85</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>5.9</v>
+        <v>10.03</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>10.69418386491559</v>
+        <v>1.827411167512683</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>6.39</v>
+        <v>10.83</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>5.526000000000001</v>
+        <v>9.582000000000001</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>5.555000000000001</v>
+        <v>9.684000000000001</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>-0.5220522052205245</v>
+        <v>-1.053283767038415</v>
       </c>
       <c r="N49" s="3" t="n">
-        <v>5.648</v>
+        <v>9.763999999999999</v>
       </c>
       <c r="O49" s="3" t="n">
-        <v>5.58</v>
+        <v>9.685</v>
       </c>
       <c r="P49" s="4" t="n">
-        <v>1.218637992831528</v>
+        <v>0.8156943727413379</v>
       </c>
       <c r="Q49" s="5" t="n">
-        <v>1.740690198052053</v>
+        <v>1.868978139779753</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
@@ -3639,56 +3639,59 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>AI应用</t>
+          <t>药</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>空</t>
-        </is>
+          <t>空转多</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>3</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>300364</t>
+          <t>300006</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>中文在线</t>
+          <t>莱美药业</t>
         </is>
       </c>
       <c r="G50" s="3" t="n">
-        <v>23.45</v>
+        <v>8.27</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>26.59</v>
+        <v>9.58</v>
       </c>
       <c r="I50" s="4" t="n">
-        <v>13.39019189765458</v>
+        <v>15.8403869407497</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>28.14</v>
+        <v>9.92</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>24.172</v>
+        <v>8.528</v>
       </c>
       <c r="L50" s="3" t="n">
-        <v>24.289</v>
+        <v>8.674000000000001</v>
       </c>
       <c r="M50" s="4" t="n">
-        <v>-0.4816995347688091</v>
+        <v>-1.683191145953433</v>
       </c>
       <c r="N50" s="3" t="n">
-        <v>24.904</v>
+        <v>8.82</v>
       </c>
       <c r="O50" s="3" t="n">
-        <v>24.422</v>
+        <v>8.818999999999999</v>
       </c>
       <c r="P50" s="4" t="n">
-        <v>1.973630333306042</v>
+        <v>0.01133915409912145</v>
       </c>
       <c r="Q50" s="5" t="n">
-        <v>2.455329868074851</v>
+        <v>1.694530300052555</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
@@ -3704,7 +3707,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>AI应用</t>
+          <t>药</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3714,46 +3717,46 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>300063</t>
+          <t>002950</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>天龙集团</t>
+          <t>奥美医疗</t>
         </is>
       </c>
       <c r="G51" s="3" t="n">
-        <v>7.93</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>9.01</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="I51" s="4" t="n">
-        <v>13.61916771752838</v>
+        <v>7.785888077858871</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>9.51</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>8.251999999999999</v>
+        <v>8.343999999999999</v>
       </c>
       <c r="L51" s="3" t="n">
-        <v>8.348000000000001</v>
+        <v>8.372</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>-1.149976042165812</v>
+        <v>-0.3344481605351279</v>
       </c>
       <c r="N51" s="3" t="n">
-        <v>8.484</v>
+        <v>8.504</v>
       </c>
       <c r="O51" s="3" t="n">
-        <v>8.375</v>
+        <v>8.406000000000001</v>
       </c>
       <c r="P51" s="4" t="n">
-        <v>1.301492537313442</v>
+        <v>1.165833928146554</v>
       </c>
       <c r="Q51" s="5" t="n">
-        <v>2.451468579479255</v>
+        <v>1.500282088681681</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
@@ -3769,7 +3772,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>AI应用</t>
+          <t>药</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3779,46 +3782,46 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>301262</t>
+          <t>301408</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>海看股份</t>
+          <t>华人健康</t>
         </is>
       </c>
       <c r="G52" s="3" t="n">
-        <v>20.35</v>
+        <v>13.78</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>23.36</v>
+        <v>14.88</v>
       </c>
       <c r="I52" s="4" t="n">
-        <v>14.79115479115478</v>
+        <v>7.982583454281578</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>24.42</v>
+        <v>16.53</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>20.914</v>
+        <v>13.936</v>
       </c>
       <c r="L52" s="3" t="n">
-        <v>21.211</v>
+        <v>13.95</v>
       </c>
       <c r="M52" s="4" t="n">
-        <v>-1.400216868605919</v>
+        <v>-0.100358422939073</v>
       </c>
       <c r="N52" s="3" t="n">
-        <v>21.638</v>
+        <v>14.236</v>
       </c>
       <c r="O52" s="3" t="n">
-        <v>21.336</v>
+        <v>14.039</v>
       </c>
       <c r="P52" s="4" t="n">
-        <v>1.415448068991365</v>
+        <v>1.403233848564733</v>
       </c>
       <c r="Q52" s="5" t="n">
-        <v>2.815664937597284</v>
+        <v>1.503592271503806</v>
       </c>
       <c r="R52" t="inlineStr">
         <is>
@@ -3834,7 +3837,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>AI应用</t>
+          <t>药</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3844,46 +3847,46 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>300959</t>
+          <t>300702</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>线上线下</t>
+          <t>天宇股份</t>
         </is>
       </c>
       <c r="G53" s="3" t="n">
-        <v>68.5</v>
+        <v>20.01</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>79.03</v>
+        <v>21.77</v>
       </c>
       <c r="I53" s="4" t="n">
-        <v>15.37226277372263</v>
+        <v>8.795602198900543</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>82.2</v>
+        <v>24.01</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>72.27799999999999</v>
+        <v>20.394</v>
       </c>
       <c r="L53" s="3" t="n">
-        <v>73.40299999999999</v>
+        <v>20.548</v>
       </c>
       <c r="M53" s="4" t="n">
-        <v>-1.532634905930275</v>
+        <v>-0.749464668094213</v>
       </c>
       <c r="N53" s="3" t="n">
-        <v>74.042</v>
+        <v>20.792</v>
       </c>
       <c r="O53" s="3" t="n">
-        <v>73.756</v>
+        <v>20.632</v>
       </c>
       <c r="P53" s="4" t="n">
-        <v>0.3877650631813001</v>
+        <v>0.7754943776657752</v>
       </c>
       <c r="Q53" s="5" t="n">
-        <v>1.920399969111575</v>
+        <v>1.524959045759988</v>
       </c>
       <c r="R53" t="inlineStr">
         <is>
@@ -3899,7 +3902,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>AI应用</t>
+          <t>药</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3909,46 +3912,46 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>300785</t>
+          <t>603259</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>值得买</t>
+          <t>药明康德</t>
         </is>
       </c>
       <c r="G54" s="3" t="n">
-        <v>32.47</v>
+        <v>141.48</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>37.95</v>
+        <v>154.19</v>
       </c>
       <c r="I54" s="4" t="n">
-        <v>16.87711733908224</v>
+        <v>8.983601922533225</v>
       </c>
       <c r="J54" s="3" t="n">
-        <v>38.96</v>
+        <v>155.62</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>34.376</v>
+        <v>145.54</v>
       </c>
       <c r="L54" s="3" t="n">
-        <v>34.82600000000001</v>
+        <v>146.801</v>
       </c>
       <c r="M54" s="4" t="n">
-        <v>-1.292138057772951</v>
+        <v>-0.8589859742099804</v>
       </c>
       <c r="N54" s="3" t="n">
-        <v>35.33</v>
+        <v>148.116</v>
       </c>
       <c r="O54" s="3" t="n">
-        <v>35.05500000000001</v>
+        <v>146.77</v>
       </c>
       <c r="P54" s="4" t="n">
-        <v>0.7844815290257934</v>
+        <v>0.9170811473734553</v>
       </c>
       <c r="Q54" s="5" t="n">
-        <v>2.076619586798745</v>
+        <v>1.776067121583436</v>
       </c>
       <c r="R54" t="inlineStr">
         <is>
@@ -3964,7 +3967,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>AI应用</t>
+          <t>药</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3974,46 +3977,46 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>301171</t>
+          <t>688710</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>易点天下</t>
+          <t>益诺思</t>
         </is>
       </c>
       <c r="G55" s="3" t="n">
-        <v>28.9</v>
+        <v>83.36</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>33.87</v>
+        <v>91.54000000000001</v>
       </c>
       <c r="I55" s="4" t="n">
-        <v>17.19723183391002</v>
+        <v>9.812859884836866</v>
       </c>
       <c r="J55" s="3" t="n">
-        <v>34.68</v>
+        <v>100.03</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>30.872</v>
+        <v>83.75</v>
       </c>
       <c r="L55" s="3" t="n">
-        <v>30.89</v>
+        <v>84.50099999999999</v>
       </c>
       <c r="M55" s="4" t="n">
-        <v>-0.0582712852055467</v>
+        <v>-0.8887468787351471</v>
       </c>
       <c r="N55" s="3" t="n">
-        <v>31.734</v>
+        <v>85.82000000000001</v>
       </c>
       <c r="O55" s="3" t="n">
-        <v>31.077</v>
+        <v>84.71000000000001</v>
       </c>
       <c r="P55" s="4" t="n">
-        <v>2.11410367796121</v>
+        <v>1.310352968952899</v>
       </c>
       <c r="Q55" s="5" t="n">
-        <v>2.172374963166757</v>
+        <v>2.199099847688046</v>
       </c>
       <c r="R55" t="inlineStr">
         <is>
@@ -4029,7 +4032,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>机器人</t>
+          <t>药</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -4039,46 +4042,46 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>301182</t>
+          <t>300363</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>凯旺科技</t>
+          <t>博腾股份</t>
         </is>
       </c>
       <c r="G56" s="3" t="n">
-        <v>43.21</v>
+        <v>20.93</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>50.56</v>
+        <v>23.15</v>
       </c>
       <c r="I56" s="4" t="n">
-        <v>17.00995140013886</v>
+        <v>10.60678451982799</v>
       </c>
       <c r="J56" s="3" t="n">
-        <v>51.85</v>
+        <v>25.11</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>46.172</v>
+        <v>21.43</v>
       </c>
       <c r="L56" s="3" t="n">
-        <v>46.638</v>
+        <v>21.526</v>
       </c>
       <c r="M56" s="4" t="n">
-        <v>-0.9991852137741675</v>
+        <v>-0.4459723125522785</v>
       </c>
       <c r="N56" s="3" t="n">
-        <v>47.264</v>
+        <v>21.876</v>
       </c>
       <c r="O56" s="3" t="n">
-        <v>46.95</v>
+        <v>21.647</v>
       </c>
       <c r="P56" s="4" t="n">
-        <v>0.6687965921192696</v>
+        <v>1.057883309465502</v>
       </c>
       <c r="Q56" s="5" t="n">
-        <v>1.667981805893437</v>
+        <v>1.50385562201778</v>
       </c>
       <c r="R56" t="inlineStr">
         <is>
@@ -4094,7 +4097,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>机器人</t>
+          <t>药</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -4104,46 +4107,46 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>688697</t>
+          <t>300255</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>纽威数控</t>
+          <t>常山药业</t>
         </is>
       </c>
       <c r="G57" s="3" t="n">
-        <v>11.76</v>
+        <v>18.73</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>13.78</v>
+        <v>20.9</v>
       </c>
       <c r="I57" s="4" t="n">
-        <v>17.17687074829932</v>
+        <v>11.58569140416443</v>
       </c>
       <c r="J57" s="3" t="n">
-        <v>14.11</v>
+        <v>22.47</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>12.474</v>
+        <v>19.526</v>
       </c>
       <c r="L57" s="3" t="n">
-        <v>12.548</v>
+        <v>19.721</v>
       </c>
       <c r="M57" s="4" t="n">
-        <v>-0.5897354160025459</v>
+        <v>-0.9887936717204893</v>
       </c>
       <c r="N57" s="3" t="n">
-        <v>12.832</v>
+        <v>19.884</v>
       </c>
       <c r="O57" s="3" t="n">
-        <v>12.656</v>
+        <v>19.782</v>
       </c>
       <c r="P57" s="4" t="n">
-        <v>1.390644753476589</v>
+        <v>0.515620260843197</v>
       </c>
       <c r="Q57" s="5" t="n">
-        <v>1.980380169479135</v>
+        <v>1.504413932563686</v>
       </c>
       <c r="R57" t="inlineStr">
         <is>
@@ -4164,54 +4167,51 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>空转多</t>
-        </is>
-      </c>
-      <c r="D58" t="n">
-        <v>3</v>
+          <t>空</t>
+        </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>300006</t>
+          <t>300705</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>莱美药业</t>
+          <t>九典制药</t>
         </is>
       </c>
       <c r="G58" s="3" t="n">
-        <v>8.27</v>
+        <v>10.33</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>9.58</v>
+        <v>11.54</v>
       </c>
       <c r="I58" s="4" t="n">
-        <v>15.8403869407497</v>
+        <v>11.71345595353339</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>9.92</v>
+        <v>12.39</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>8.528</v>
+        <v>10.682</v>
       </c>
       <c r="L58" s="3" t="n">
-        <v>8.674000000000001</v>
+        <v>10.718</v>
       </c>
       <c r="M58" s="4" t="n">
-        <v>-1.683191145953433</v>
+        <v>-0.3358835603657573</v>
       </c>
       <c r="N58" s="3" t="n">
-        <v>8.82</v>
+        <v>10.926</v>
       </c>
       <c r="O58" s="3" t="n">
-        <v>8.818999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="P58" s="4" t="n">
-        <v>0.01133915409912145</v>
+        <v>1.166666666666649</v>
       </c>
       <c r="Q58" s="5" t="n">
-        <v>1.694530300052555</v>
+        <v>1.502550227032406</v>
       </c>
       <c r="R58" t="inlineStr">
         <is>
@@ -4237,46 +4237,46 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>002950</t>
+          <t>688607</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>奥美医疗</t>
+          <t>康众科技</t>
         </is>
       </c>
       <c r="G59" s="3" t="n">
-        <v>8.220000000000001</v>
+        <v>31</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>8.859999999999999</v>
+        <v>34.67</v>
       </c>
       <c r="I59" s="4" t="n">
-        <v>7.785888077858871</v>
+        <v>11.83870967741936</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>9.039999999999999</v>
+        <v>37.2</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>8.343999999999999</v>
+        <v>32.822</v>
       </c>
       <c r="L59" s="3" t="n">
-        <v>8.372</v>
+        <v>33.042</v>
       </c>
       <c r="M59" s="4" t="n">
-        <v>-0.3344481605351279</v>
+        <v>-0.6658192603353319</v>
       </c>
       <c r="N59" s="3" t="n">
-        <v>8.504</v>
+        <v>33.384</v>
       </c>
       <c r="O59" s="3" t="n">
-        <v>8.406000000000001</v>
+        <v>33.10700000000001</v>
       </c>
       <c r="P59" s="4" t="n">
-        <v>1.165833928146554</v>
+        <v>0.8366810644274469</v>
       </c>
       <c r="Q59" s="5" t="n">
-        <v>1.500282088681681</v>
+        <v>1.502500324762779</v>
       </c>
       <c r="R59" t="inlineStr">
         <is>
@@ -4302,46 +4302,46 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>301408</t>
+          <t>300434</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>华人健康</t>
+          <t>金石亚药</t>
         </is>
       </c>
       <c r="G60" s="3" t="n">
-        <v>13.78</v>
+        <v>11.31</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>14.88</v>
+        <v>12.66</v>
       </c>
       <c r="I60" s="4" t="n">
-        <v>7.982583454281578</v>
+        <v>11.93633952254642</v>
       </c>
       <c r="J60" s="3" t="n">
-        <v>16.53</v>
+        <v>13.57</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>13.936</v>
+        <v>12.044</v>
       </c>
       <c r="L60" s="3" t="n">
-        <v>13.95</v>
+        <v>12.294</v>
       </c>
       <c r="M60" s="4" t="n">
-        <v>-0.100358422939073</v>
+        <v>-2.033512282414185</v>
       </c>
       <c r="N60" s="3" t="n">
-        <v>14.236</v>
+        <v>12.242</v>
       </c>
       <c r="O60" s="3" t="n">
-        <v>14.039</v>
+        <v>12.24</v>
       </c>
       <c r="P60" s="4" t="n">
-        <v>1.403233848564733</v>
+        <v>0.01633986928104569</v>
       </c>
       <c r="Q60" s="5" t="n">
-        <v>1.503592271503806</v>
+        <v>2.049852151695231</v>
       </c>
       <c r="R60" t="inlineStr">
         <is>
@@ -4367,46 +4367,46 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>300702</t>
+          <t>301277</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>天宇股份</t>
+          <t>新天地</t>
         </is>
       </c>
       <c r="G61" s="3" t="n">
-        <v>20.01</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>21.77</v>
+        <v>10.34</v>
       </c>
       <c r="I61" s="4" t="n">
-        <v>8.795602198900543</v>
+        <v>12.14750542299348</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>24.01</v>
+        <v>11.06</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>20.394</v>
+        <v>9.634</v>
       </c>
       <c r="L61" s="3" t="n">
-        <v>20.548</v>
+        <v>9.775000000000002</v>
       </c>
       <c r="M61" s="4" t="n">
-        <v>-0.749464668094213</v>
+        <v>-1.442455242966767</v>
       </c>
       <c r="N61" s="3" t="n">
-        <v>20.792</v>
+        <v>9.818000000000001</v>
       </c>
       <c r="O61" s="3" t="n">
-        <v>20.632</v>
+        <v>9.792000000000002</v>
       </c>
       <c r="P61" s="4" t="n">
-        <v>0.7754943776657752</v>
+        <v>0.2655228758169814</v>
       </c>
       <c r="Q61" s="5" t="n">
-        <v>1.524959045759988</v>
+        <v>1.707978118783748</v>
       </c>
       <c r="R61" t="inlineStr">
         <is>
@@ -4432,46 +4432,46 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>603259</t>
+          <t>301333</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>药明康德</t>
+          <t>诺思格</t>
         </is>
       </c>
       <c r="G62" s="3" t="n">
-        <v>141.48</v>
+        <v>51.85</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>154.19</v>
+        <v>58.46</v>
       </c>
       <c r="I62" s="4" t="n">
-        <v>8.983601922533225</v>
+        <v>12.74831243972998</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>155.62</v>
+        <v>62.22</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>145.54</v>
+        <v>53.51000000000001</v>
       </c>
       <c r="L62" s="3" t="n">
-        <v>146.801</v>
+        <v>54.26900000000001</v>
       </c>
       <c r="M62" s="4" t="n">
-        <v>-0.8589859742099804</v>
+        <v>-1.398588512778931</v>
       </c>
       <c r="N62" s="3" t="n">
-        <v>148.116</v>
+        <v>54.876</v>
       </c>
       <c r="O62" s="3" t="n">
-        <v>146.77</v>
+        <v>54.463</v>
       </c>
       <c r="P62" s="4" t="n">
-        <v>0.9170811473734553</v>
+        <v>0.7583129831261637</v>
       </c>
       <c r="Q62" s="5" t="n">
-        <v>1.776067121583436</v>
+        <v>2.156901495905095</v>
       </c>
       <c r="R62" t="inlineStr">
         <is>
@@ -4497,46 +4497,46 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>600479</t>
+          <t>300246</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>XD千金药</t>
+          <t>宝莱特</t>
         </is>
       </c>
       <c r="G63" s="3" t="n">
-        <v>10.46</v>
+        <v>12.22</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>11.42</v>
+        <v>13.85</v>
       </c>
       <c r="I63" s="4" t="n">
-        <v>9.17782026768641</v>
+        <v>13.33878887070377</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>11.5</v>
+        <v>14.66</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>10.754</v>
+        <v>12.864</v>
       </c>
       <c r="L63" s="3" t="n">
-        <v>10.879</v>
+        <v>12.941</v>
       </c>
       <c r="M63" s="4" t="n">
-        <v>-1.149002665686183</v>
+        <v>-0.5950081137470087</v>
       </c>
       <c r="N63" s="3" t="n">
-        <v>10.928</v>
+        <v>13.106</v>
       </c>
       <c r="O63" s="3" t="n">
-        <v>10.889</v>
+        <v>12.988</v>
       </c>
       <c r="P63" s="4" t="n">
-        <v>0.3581596106162044</v>
+        <v>0.9085309516476681</v>
       </c>
       <c r="Q63" s="5" t="n">
-        <v>1.507162276302387</v>
+        <v>1.503539065394677</v>
       </c>
       <c r="R63" t="inlineStr">
         <is>
@@ -4562,46 +4562,46 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>688710</t>
+          <t>300109</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>益诺思</t>
+          <t>新开源</t>
         </is>
       </c>
       <c r="G64" s="3" t="n">
-        <v>83.36</v>
+        <v>10.77</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>91.54000000000001</v>
+        <v>12.33</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>9.812859884836866</v>
+        <v>14.48467966573816</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>100.03</v>
+        <v>12.92</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>83.75</v>
+        <v>11.36</v>
       </c>
       <c r="L64" s="3" t="n">
-        <v>84.50099999999999</v>
+        <v>11.514</v>
       </c>
       <c r="M64" s="4" t="n">
-        <v>-0.8887468787351471</v>
+        <v>-1.337502171269755</v>
       </c>
       <c r="N64" s="3" t="n">
-        <v>85.82000000000001</v>
+        <v>11.602</v>
       </c>
       <c r="O64" s="3" t="n">
-        <v>84.71000000000001</v>
+        <v>11.577</v>
       </c>
       <c r="P64" s="4" t="n">
-        <v>1.310352968952899</v>
+        <v>0.2159454090005841</v>
       </c>
       <c r="Q64" s="5" t="n">
-        <v>2.199099847688046</v>
+        <v>1.55344758027034</v>
       </c>
       <c r="R64" t="inlineStr">
         <is>
@@ -4627,46 +4627,46 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>300363</t>
+          <t>300347</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>博腾股份</t>
+          <t>泰格医药</t>
         </is>
       </c>
       <c r="G65" s="3" t="n">
-        <v>20.93</v>
+        <v>47.82</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>23.15</v>
+        <v>54.89</v>
       </c>
       <c r="I65" s="4" t="n">
-        <v>10.60678451982799</v>
+        <v>14.78460895023004</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>25.11</v>
+        <v>57.38</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>21.43</v>
+        <v>50.25599999999999</v>
       </c>
       <c r="L65" s="3" t="n">
-        <v>21.526</v>
+        <v>50.69799999999999</v>
       </c>
       <c r="M65" s="4" t="n">
-        <v>-0.4459723125522785</v>
+        <v>-0.8718292634817937</v>
       </c>
       <c r="N65" s="3" t="n">
-        <v>21.876</v>
+        <v>51.302</v>
       </c>
       <c r="O65" s="3" t="n">
-        <v>21.647</v>
+        <v>50.98099999999999</v>
       </c>
       <c r="P65" s="4" t="n">
-        <v>1.057883309465502</v>
+        <v>0.6296463388321349</v>
       </c>
       <c r="Q65" s="5" t="n">
-        <v>1.50385562201778</v>
+        <v>1.501475602313929</v>
       </c>
       <c r="R65" t="inlineStr">
         <is>
@@ -4692,46 +4692,46 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>300255</t>
+          <t>300723</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>常山药业</t>
+          <t>一品红</t>
         </is>
       </c>
       <c r="G66" s="3" t="n">
-        <v>18.73</v>
+        <v>28.77</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>20.9</v>
+        <v>33.08</v>
       </c>
       <c r="I66" s="4" t="n">
-        <v>11.58569140416443</v>
+        <v>14.98088286409454</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>22.47</v>
+        <v>34.52</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>19.526</v>
+        <v>30.38</v>
       </c>
       <c r="L66" s="3" t="n">
-        <v>19.721</v>
+        <v>30.584</v>
       </c>
       <c r="M66" s="4" t="n">
-        <v>-0.9887936717204893</v>
+        <v>-0.6670154329060929</v>
       </c>
       <c r="N66" s="3" t="n">
-        <v>19.884</v>
+        <v>31.088</v>
       </c>
       <c r="O66" s="3" t="n">
-        <v>19.782</v>
+        <v>30.831</v>
       </c>
       <c r="P66" s="4" t="n">
-        <v>0.515620260843197</v>
+        <v>0.8335765949855745</v>
       </c>
       <c r="Q66" s="5" t="n">
-        <v>1.504413932563686</v>
+        <v>1.500592027891667</v>
       </c>
       <c r="R66" t="inlineStr">
         <is>
@@ -4757,46 +4757,46 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>300705</t>
+          <t>300683</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>九典制药</t>
+          <t>海特生物</t>
         </is>
       </c>
       <c r="G67" s="3" t="n">
-        <v>10.33</v>
+        <v>21.76</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>11.54</v>
+        <v>25.03</v>
       </c>
       <c r="I67" s="4" t="n">
-        <v>11.71345595353339</v>
+        <v>15.02757352941175</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>12.39</v>
+        <v>26.11</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>10.682</v>
+        <v>23.268</v>
       </c>
       <c r="L67" s="3" t="n">
-        <v>10.718</v>
+        <v>23.612</v>
       </c>
       <c r="M67" s="4" t="n">
-        <v>-0.3358835603657573</v>
+        <v>-1.456886328985241</v>
       </c>
       <c r="N67" s="3" t="n">
-        <v>10.926</v>
+        <v>23.674</v>
       </c>
       <c r="O67" s="3" t="n">
-        <v>10.8</v>
+        <v>23.663</v>
       </c>
       <c r="P67" s="4" t="n">
-        <v>1.166666666666649</v>
+        <v>0.0464860753074392</v>
       </c>
       <c r="Q67" s="5" t="n">
-        <v>1.502550227032406</v>
+        <v>1.50337240429268</v>
       </c>
       <c r="R67" t="inlineStr">
         <is>
@@ -4822,46 +4822,46 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>688607</t>
+          <t>300725</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>康众科技</t>
+          <t>药石科技</t>
         </is>
       </c>
       <c r="G68" s="3" t="n">
-        <v>31</v>
+        <v>41.36</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>34.67</v>
+        <v>47.86</v>
       </c>
       <c r="I68" s="4" t="n">
-        <v>11.83870967741936</v>
+        <v>15.71566731141198</v>
       </c>
       <c r="J68" s="3" t="n">
-        <v>37.2</v>
+        <v>49.63</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>32.822</v>
+        <v>44.188</v>
       </c>
       <c r="L68" s="3" t="n">
-        <v>33.042</v>
+        <v>44.511</v>
       </c>
       <c r="M68" s="4" t="n">
-        <v>-0.6658192603353319</v>
+        <v>-0.7256633191795259</v>
       </c>
       <c r="N68" s="3" t="n">
-        <v>33.384</v>
+        <v>45.09999999999999</v>
       </c>
       <c r="O68" s="3" t="n">
-        <v>33.10700000000001</v>
+        <v>44.753</v>
       </c>
       <c r="P68" s="4" t="n">
-        <v>0.8366810644274469</v>
+        <v>0.7753670145018043</v>
       </c>
       <c r="Q68" s="5" t="n">
-        <v>1.502500324762779</v>
+        <v>1.50103033368133</v>
       </c>
       <c r="R68" t="inlineStr">
         <is>
@@ -4887,46 +4887,46 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>300434</t>
+          <t>301257</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>金石亚药</t>
+          <t>普蕊斯</t>
         </is>
       </c>
       <c r="G69" s="3" t="n">
-        <v>11.31</v>
+        <v>31.5</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>12.66</v>
+        <v>36.68</v>
       </c>
       <c r="I69" s="4" t="n">
-        <v>11.93633952254642</v>
+        <v>16.44444444444444</v>
       </c>
       <c r="J69" s="3" t="n">
-        <v>13.57</v>
+        <v>37.8</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>12.044</v>
+        <v>33.264</v>
       </c>
       <c r="L69" s="3" t="n">
-        <v>12.294</v>
+        <v>33.722</v>
       </c>
       <c r="M69" s="4" t="n">
-        <v>-2.033512282414185</v>
+        <v>-1.358163809975699</v>
       </c>
       <c r="N69" s="3" t="n">
-        <v>12.242</v>
+        <v>34.134</v>
       </c>
       <c r="O69" s="3" t="n">
-        <v>12.24</v>
+        <v>33.854</v>
       </c>
       <c r="P69" s="4" t="n">
-        <v>0.01633986928104569</v>
+        <v>0.8270809948602853</v>
       </c>
       <c r="Q69" s="5" t="n">
-        <v>2.049852151695231</v>
+        <v>2.185244804835984</v>
       </c>
       <c r="R69" t="inlineStr">
         <is>
@@ -4952,46 +4952,46 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>301277</t>
+          <t>301093</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>新天地</t>
+          <t>华兰股份</t>
         </is>
       </c>
       <c r="G70" s="3" t="n">
-        <v>9.220000000000001</v>
+        <v>47.68</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>10.34</v>
+        <v>55.64</v>
       </c>
       <c r="I70" s="4" t="n">
-        <v>12.14750542299348</v>
+        <v>16.69463087248322</v>
       </c>
       <c r="J70" s="3" t="n">
-        <v>11.06</v>
+        <v>57.21</v>
       </c>
       <c r="K70" s="3" t="n">
-        <v>9.634</v>
+        <v>50.5</v>
       </c>
       <c r="L70" s="3" t="n">
-        <v>9.775000000000002</v>
+        <v>51.384</v>
       </c>
       <c r="M70" s="4" t="n">
-        <v>-1.442455242966767</v>
+        <v>-1.720379884789036</v>
       </c>
       <c r="N70" s="3" t="n">
-        <v>9.818000000000001</v>
+        <v>51.824</v>
       </c>
       <c r="O70" s="3" t="n">
-        <v>9.792000000000002</v>
+        <v>51.822</v>
       </c>
       <c r="P70" s="4" t="n">
-        <v>0.2655228758169814</v>
+        <v>0.003859364748559635</v>
       </c>
       <c r="Q70" s="5" t="n">
-        <v>1.707978118783748</v>
+        <v>1.724239249537596</v>
       </c>
       <c r="R70" t="inlineStr">
         <is>
@@ -5017,46 +5017,46 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>301333</t>
+          <t>301201</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>诺思格</t>
+          <t>诚达药业</t>
         </is>
       </c>
       <c r="G71" s="3" t="n">
-        <v>51.85</v>
+        <v>24.01</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>58.46</v>
+        <v>28.02</v>
       </c>
       <c r="I71" s="4" t="n">
-        <v>12.74831243972998</v>
+        <v>16.70137442732194</v>
       </c>
       <c r="J71" s="3" t="n">
-        <v>62.22</v>
+        <v>28.81</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>53.51000000000001</v>
+        <v>25.546</v>
       </c>
       <c r="L71" s="3" t="n">
-        <v>54.26900000000001</v>
+        <v>25.963</v>
       </c>
       <c r="M71" s="4" t="n">
-        <v>-1.398588512778931</v>
+        <v>-1.606131802950361</v>
       </c>
       <c r="N71" s="3" t="n">
-        <v>54.876</v>
+        <v>26.066</v>
       </c>
       <c r="O71" s="3" t="n">
-        <v>54.463</v>
+        <v>26.065</v>
       </c>
       <c r="P71" s="4" t="n">
-        <v>0.7583129831261637</v>
+        <v>0.003836562440051594</v>
       </c>
       <c r="Q71" s="5" t="n">
-        <v>2.156901495905095</v>
+        <v>1.609968365390413</v>
       </c>
       <c r="R71" t="inlineStr">
         <is>
@@ -5082,46 +5082,46 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>300246</t>
+          <t>920047</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>宝莱特</t>
+          <t>诺思兰德</t>
         </is>
       </c>
       <c r="G72" s="3" t="n">
-        <v>12.22</v>
+        <v>12.62</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>13.85</v>
+        <v>14.75</v>
       </c>
       <c r="I72" s="4" t="n">
-        <v>13.33878887070377</v>
+        <v>16.87797147385104</v>
       </c>
       <c r="J72" s="3" t="n">
-        <v>14.66</v>
+        <v>15.14</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>12.864</v>
+        <v>13.434</v>
       </c>
       <c r="L72" s="3" t="n">
-        <v>12.941</v>
+        <v>13.55</v>
       </c>
       <c r="M72" s="4" t="n">
-        <v>-0.5950081137470087</v>
+        <v>-0.8560885608856372</v>
       </c>
       <c r="N72" s="3" t="n">
-        <v>13.106</v>
+        <v>13.722</v>
       </c>
       <c r="O72" s="3" t="n">
-        <v>12.988</v>
+        <v>13.634</v>
       </c>
       <c r="P72" s="4" t="n">
-        <v>0.9085309516476681</v>
+        <v>0.6454452105031372</v>
       </c>
       <c r="Q72" s="5" t="n">
-        <v>1.503539065394677</v>
+        <v>1.501533771388774</v>
       </c>
       <c r="R72" t="inlineStr">
         <is>
@@ -5147,46 +5147,46 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>300109</t>
+          <t>300204</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>新开源</t>
+          <t>舒泰神</t>
         </is>
       </c>
       <c r="G73" s="3" t="n">
-        <v>10.77</v>
+        <v>16.91</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>12.33</v>
+        <v>19.8</v>
       </c>
       <c r="I73" s="4" t="n">
-        <v>14.48467966573816</v>
+        <v>17.09047900650502</v>
       </c>
       <c r="J73" s="3" t="n">
-        <v>12.92</v>
+        <v>20.29</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>11.36</v>
+        <v>17.97</v>
       </c>
       <c r="L73" s="3" t="n">
-        <v>11.514</v>
+        <v>18.211</v>
       </c>
       <c r="M73" s="4" t="n">
-        <v>-1.337502171269755</v>
+        <v>-1.323375981549613</v>
       </c>
       <c r="N73" s="3" t="n">
-        <v>11.602</v>
+        <v>18.47</v>
       </c>
       <c r="O73" s="3" t="n">
-        <v>11.577</v>
+        <v>18.264</v>
       </c>
       <c r="P73" s="4" t="n">
-        <v>0.2159454090005841</v>
+        <v>1.127901883486615</v>
       </c>
       <c r="Q73" s="5" t="n">
-        <v>1.55344758027034</v>
+        <v>2.451277865036228</v>
       </c>
       <c r="R73" t="inlineStr">
         <is>
@@ -5212,46 +5212,46 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>300347</t>
+          <t>300534</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>泰格医药</t>
+          <t>陇神戎发</t>
         </is>
       </c>
       <c r="G74" s="3" t="n">
-        <v>47.82</v>
+        <v>9.68</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>54.89</v>
+        <v>11.41</v>
       </c>
       <c r="I74" s="4" t="n">
-        <v>14.78460895023004</v>
+        <v>17.8719008264463</v>
       </c>
       <c r="J74" s="3" t="n">
-        <v>57.38</v>
+        <v>11.61</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>50.25599999999999</v>
+        <v>10.302</v>
       </c>
       <c r="L74" s="3" t="n">
-        <v>50.69799999999999</v>
+        <v>10.524</v>
       </c>
       <c r="M74" s="4" t="n">
-        <v>-0.8718292634817937</v>
+        <v>-2.109464082098089</v>
       </c>
       <c r="N74" s="3" t="n">
-        <v>51.302</v>
+        <v>10.564</v>
       </c>
       <c r="O74" s="3" t="n">
-        <v>50.98099999999999</v>
+        <v>10.562</v>
       </c>
       <c r="P74" s="4" t="n">
-        <v>0.6296463388321349</v>
+        <v>0.01893580761218594</v>
       </c>
       <c r="Q74" s="5" t="n">
-        <v>1.501475602313929</v>
+        <v>2.128399889710275</v>
       </c>
       <c r="R74" t="inlineStr">
         <is>
@@ -5277,46 +5277,46 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>300723</t>
+          <t>300436</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>一品红</t>
+          <t>广生堂</t>
         </is>
       </c>
       <c r="G75" s="3" t="n">
-        <v>28.77</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>33.08</v>
+        <v>83.91</v>
       </c>
       <c r="I75" s="4" t="n">
-        <v>14.98088286409454</v>
+        <v>18.34978843441466</v>
       </c>
       <c r="J75" s="3" t="n">
-        <v>34.52</v>
+        <v>85.08</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>30.38</v>
+        <v>76.474</v>
       </c>
       <c r="L75" s="3" t="n">
-        <v>30.584</v>
+        <v>77.93899999999999</v>
       </c>
       <c r="M75" s="4" t="n">
-        <v>-0.6670154329060929</v>
+        <v>-1.879675130550806</v>
       </c>
       <c r="N75" s="3" t="n">
-        <v>31.088</v>
+        <v>78.164</v>
       </c>
       <c r="O75" s="3" t="n">
-        <v>30.831</v>
+        <v>78.16199999999999</v>
       </c>
       <c r="P75" s="4" t="n">
-        <v>0.8335765949855745</v>
+        <v>0.002558788157935865</v>
       </c>
       <c r="Q75" s="5" t="n">
-        <v>1.500592027891667</v>
+        <v>1.882233918708742</v>
       </c>
       <c r="R75" t="inlineStr">
         <is>
@@ -5342,46 +5342,46 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>300683</t>
+          <t>301234</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>海特生物</t>
+          <t>五洲医疗</t>
         </is>
       </c>
       <c r="G76" s="3" t="n">
-        <v>21.76</v>
+        <v>125.7</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>25.03</v>
+        <v>149.04</v>
       </c>
       <c r="I76" s="4" t="n">
-        <v>15.02757352941175</v>
+        <v>18.56801909307875</v>
       </c>
       <c r="J76" s="3" t="n">
-        <v>26.11</v>
+        <v>150.84</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>23.268</v>
+        <v>130.836</v>
       </c>
       <c r="L76" s="3" t="n">
-        <v>23.612</v>
+        <v>131.754</v>
       </c>
       <c r="M76" s="4" t="n">
-        <v>-1.456886328985241</v>
+        <v>-0.6967530397559152</v>
       </c>
       <c r="N76" s="3" t="n">
-        <v>23.674</v>
+        <v>134.844</v>
       </c>
       <c r="O76" s="3" t="n">
-        <v>23.663</v>
+        <v>132.851</v>
       </c>
       <c r="P76" s="4" t="n">
-        <v>0.0464860753074392</v>
+        <v>1.50017688989923</v>
       </c>
       <c r="Q76" s="5" t="n">
-        <v>1.50337240429268</v>
+        <v>2.196929929655145</v>
       </c>
       <c r="R76" t="inlineStr">
         <is>
@@ -5407,46 +5407,46 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>300725</t>
+          <t>920367</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>药石科技</t>
+          <t>新赣江</t>
         </is>
       </c>
       <c r="G77" s="3" t="n">
-        <v>41.36</v>
+        <v>19.95</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>47.86</v>
+        <v>23.8</v>
       </c>
       <c r="I77" s="4" t="n">
-        <v>15.71566731141198</v>
+        <v>19.2982456140351</v>
       </c>
       <c r="J77" s="3" t="n">
-        <v>49.63</v>
+        <v>23.94</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>44.188</v>
+        <v>21.502</v>
       </c>
       <c r="L77" s="3" t="n">
-        <v>44.511</v>
+        <v>21.968</v>
       </c>
       <c r="M77" s="4" t="n">
-        <v>-0.7256633191795259</v>
+        <v>-2.12126729788783</v>
       </c>
       <c r="N77" s="3" t="n">
-        <v>45.09999999999999</v>
+        <v>22.098</v>
       </c>
       <c r="O77" s="3" t="n">
-        <v>44.753</v>
+        <v>21.968</v>
       </c>
       <c r="P77" s="4" t="n">
-        <v>0.7753670145018043</v>
+        <v>0.5917698470502719</v>
       </c>
       <c r="Q77" s="5" t="n">
-        <v>1.50103033368133</v>
+        <v>2.713037144938102</v>
       </c>
       <c r="R77" t="inlineStr">
         <is>
@@ -5462,56 +5462,59 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>药</t>
+          <t>互金证券</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>空</t>
-        </is>
+          <t>空转多</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>1</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>301257</t>
+          <t>601211</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>普蕊斯</t>
+          <t>国泰海通</t>
         </is>
       </c>
       <c r="G78" s="3" t="n">
-        <v>31.5</v>
+        <v>16.27</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>36.68</v>
+        <v>17.35</v>
       </c>
       <c r="I78" s="4" t="n">
-        <v>16.44444444444444</v>
+        <v>6.637984019668108</v>
       </c>
       <c r="J78" s="3" t="n">
-        <v>37.8</v>
+        <v>17.89</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>33.264</v>
+        <v>16.44</v>
       </c>
       <c r="L78" s="3" t="n">
-        <v>33.722</v>
+        <v>16.454</v>
       </c>
       <c r="M78" s="4" t="n">
-        <v>-1.358163809975699</v>
+        <v>-0.08508569344841677</v>
       </c>
       <c r="N78" s="3" t="n">
-        <v>34.134</v>
+        <v>16.728</v>
       </c>
       <c r="O78" s="3" t="n">
-        <v>33.854</v>
+        <v>16.494</v>
       </c>
       <c r="P78" s="4" t="n">
-        <v>0.8270809948602853</v>
+        <v>1.418697708257555</v>
       </c>
       <c r="Q78" s="5" t="n">
-        <v>2.185244804835984</v>
+        <v>1.503783401705971</v>
       </c>
       <c r="R78" t="inlineStr">
         <is>
@@ -5527,56 +5530,59 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>药</t>
+          <t>互金证券</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>空</t>
-        </is>
+          <t>空转多</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>3</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>301093</t>
+          <t>600621</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>华兰股份</t>
+          <t>华鑫股份</t>
         </is>
       </c>
       <c r="G79" s="3" t="n">
-        <v>47.68</v>
+        <v>14.9</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>55.64</v>
+        <v>15.91</v>
       </c>
       <c r="I79" s="4" t="n">
-        <v>16.69463087248322</v>
+        <v>6.778523489932886</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>57.21</v>
+        <v>16.39</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>50.5</v>
+        <v>14.66</v>
       </c>
       <c r="L79" s="3" t="n">
-        <v>51.384</v>
+        <v>14.77</v>
       </c>
       <c r="M79" s="4" t="n">
-        <v>-1.720379884789036</v>
+        <v>-0.7447528774542911</v>
       </c>
       <c r="N79" s="3" t="n">
-        <v>51.824</v>
+        <v>14.996</v>
       </c>
       <c r="O79" s="3" t="n">
-        <v>51.822</v>
+        <v>14.883</v>
       </c>
       <c r="P79" s="4" t="n">
-        <v>0.003859364748559635</v>
+        <v>0.7592555264395617</v>
       </c>
       <c r="Q79" s="5" t="n">
-        <v>1.724239249537596</v>
+        <v>1.504008403893853</v>
       </c>
       <c r="R79" t="inlineStr">
         <is>
@@ -5592,7 +5598,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>药</t>
+          <t>互金证券</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -5602,46 +5608,46 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>301201</t>
+          <t>601519</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>诚达药业</t>
+          <t>大智慧</t>
         </is>
       </c>
       <c r="G80" s="3" t="n">
-        <v>24.01</v>
+        <v>8.76</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>28.02</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="I80" s="4" t="n">
-        <v>16.70137442732194</v>
+        <v>7.191780821917826</v>
       </c>
       <c r="J80" s="3" t="n">
-        <v>28.81</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>25.546</v>
+        <v>9.022</v>
       </c>
       <c r="L80" s="3" t="n">
-        <v>25.963</v>
+        <v>9.144000000000002</v>
       </c>
       <c r="M80" s="4" t="n">
-        <v>-1.606131802950361</v>
+        <v>-1.334208223972022</v>
       </c>
       <c r="N80" s="3" t="n">
-        <v>26.066</v>
+        <v>9.218</v>
       </c>
       <c r="O80" s="3" t="n">
-        <v>26.065</v>
+        <v>9.118</v>
       </c>
       <c r="P80" s="4" t="n">
-        <v>0.003836562440051594</v>
+        <v>1.096731739416534</v>
       </c>
       <c r="Q80" s="5" t="n">
-        <v>1.609968365390413</v>
+        <v>2.430939963388556</v>
       </c>
       <c r="R80" t="inlineStr">
         <is>
@@ -5657,7 +5663,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>药</t>
+          <t>互金证券</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -5667,46 +5673,46 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>920047</t>
+          <t>600958</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>诺思兰德</t>
+          <t>东方证券</t>
         </is>
       </c>
       <c r="G81" s="3" t="n">
-        <v>12.62</v>
+        <v>8.48</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>14.75</v>
+        <v>9.15</v>
       </c>
       <c r="I81" s="4" t="n">
-        <v>16.87797147385104</v>
+        <v>7.900943396226423</v>
       </c>
       <c r="J81" s="3" t="n">
-        <v>15.14</v>
+        <v>9.32</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>13.434</v>
+        <v>8.586</v>
       </c>
       <c r="L81" s="3" t="n">
-        <v>13.55</v>
+        <v>8.595000000000002</v>
       </c>
       <c r="M81" s="4" t="n">
-        <v>-0.8560885608856372</v>
+        <v>-0.1047120418848468</v>
       </c>
       <c r="N81" s="3" t="n">
-        <v>13.722</v>
+        <v>8.75</v>
       </c>
       <c r="O81" s="3" t="n">
-        <v>13.634</v>
+        <v>8.629</v>
       </c>
       <c r="P81" s="4" t="n">
-        <v>0.6454452105031372</v>
+        <v>1.402248232703673</v>
       </c>
       <c r="Q81" s="5" t="n">
-        <v>1.501533771388774</v>
+        <v>1.50696027458852</v>
       </c>
       <c r="R81" t="inlineStr">
         <is>
@@ -5722,7 +5728,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>药</t>
+          <t>互金证券</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -5732,46 +5738,46 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>300204</t>
+          <t>601377</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>舒泰神</t>
+          <t>兴业证券</t>
         </is>
       </c>
       <c r="G82" s="3" t="n">
-        <v>16.91</v>
+        <v>5.52</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>19.8</v>
+        <v>6</v>
       </c>
       <c r="I82" s="4" t="n">
-        <v>17.09047900650502</v>
+        <v>8.695652173913061</v>
       </c>
       <c r="J82" s="3" t="n">
-        <v>20.29</v>
+        <v>6.07</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>17.97</v>
+        <v>5.613999999999999</v>
       </c>
       <c r="L82" s="3" t="n">
-        <v>18.211</v>
+        <v>5.625999999999999</v>
       </c>
       <c r="M82" s="4" t="n">
-        <v>-1.323375981549613</v>
+        <v>-0.2132954141486065</v>
       </c>
       <c r="N82" s="3" t="n">
-        <v>18.47</v>
+        <v>5.726</v>
       </c>
       <c r="O82" s="3" t="n">
-        <v>18.264</v>
+        <v>5.653</v>
       </c>
       <c r="P82" s="4" t="n">
-        <v>1.127901883486615</v>
+        <v>1.291349725809288</v>
       </c>
       <c r="Q82" s="5" t="n">
-        <v>2.451277865036228</v>
+        <v>1.504645139957894</v>
       </c>
       <c r="R82" t="inlineStr">
         <is>
@@ -5787,7 +5793,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>药</t>
+          <t>互金证券</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -5797,46 +5803,46 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>300534</t>
+          <t>002736</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>陇神戎发</t>
+          <t>国信证券</t>
         </is>
       </c>
       <c r="G83" s="3" t="n">
-        <v>9.68</v>
+        <v>9.66</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>11.41</v>
+        <v>10.52</v>
       </c>
       <c r="I83" s="4" t="n">
-        <v>17.8719008264463</v>
+        <v>8.902691511387161</v>
       </c>
       <c r="J83" s="3" t="n">
-        <v>11.61</v>
+        <v>10.62</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>10.302</v>
+        <v>9.806000000000001</v>
       </c>
       <c r="L83" s="3" t="n">
-        <v>10.524</v>
+        <v>9.812999999999999</v>
       </c>
       <c r="M83" s="4" t="n">
-        <v>-2.109464082098089</v>
+        <v>-0.07133394476712684</v>
       </c>
       <c r="N83" s="3" t="n">
-        <v>10.564</v>
+        <v>10.008</v>
       </c>
       <c r="O83" s="3" t="n">
-        <v>10.562</v>
+        <v>9.866999999999999</v>
       </c>
       <c r="P83" s="4" t="n">
-        <v>0.01893580761218594</v>
+        <v>1.429005776831871</v>
       </c>
       <c r="Q83" s="5" t="n">
-        <v>2.128399889710275</v>
+        <v>1.500339721598998</v>
       </c>
       <c r="R83" t="inlineStr">
         <is>
@@ -5852,7 +5858,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>药</t>
+          <t>互金证券</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -5862,46 +5868,46 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>300436</t>
+          <t>601136</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>广生堂</t>
+          <t>首创证券</t>
         </is>
       </c>
       <c r="G84" s="3" t="n">
-        <v>70.90000000000001</v>
+        <v>13.49</v>
       </c>
       <c r="H84" s="3" t="n">
-        <v>83.91</v>
+        <v>14.78</v>
       </c>
       <c r="I84" s="4" t="n">
-        <v>18.34978843441466</v>
+        <v>9.562638991845795</v>
       </c>
       <c r="J84" s="3" t="n">
-        <v>85.08</v>
+        <v>14.83</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>76.474</v>
+        <v>13.94</v>
       </c>
       <c r="L84" s="3" t="n">
-        <v>77.93899999999999</v>
+        <v>14.029</v>
       </c>
       <c r="M84" s="4" t="n">
-        <v>-1.879675130550806</v>
+        <v>-0.6344001710741898</v>
       </c>
       <c r="N84" s="3" t="n">
-        <v>78.164</v>
+        <v>14.184</v>
       </c>
       <c r="O84" s="3" t="n">
-        <v>78.16199999999999</v>
+        <v>14.062</v>
       </c>
       <c r="P84" s="4" t="n">
-        <v>0.002558788157935865</v>
+        <v>0.8675864030721181</v>
       </c>
       <c r="Q84" s="5" t="n">
-        <v>1.882233918708742</v>
+        <v>1.501986574146308</v>
       </c>
       <c r="R84" t="inlineStr">
         <is>
@@ -5917,7 +5923,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>药</t>
+          <t>互金证券</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -5927,46 +5933,46 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>301234</t>
+          <t>688318</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>五洲医疗</t>
+          <t>财富趋势</t>
         </is>
       </c>
       <c r="G85" s="3" t="n">
-        <v>125.7</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H85" s="3" t="n">
-        <v>149.04</v>
+        <v>77.61</v>
       </c>
       <c r="I85" s="4" t="n">
-        <v>18.56801909307875</v>
+        <v>10.88726960994428</v>
       </c>
       <c r="J85" s="3" t="n">
-        <v>150.84</v>
+        <v>83.98</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>130.836</v>
+        <v>73.66400000000002</v>
       </c>
       <c r="L85" s="3" t="n">
-        <v>131.754</v>
+        <v>73.70700000000001</v>
       </c>
       <c r="M85" s="4" t="n">
-        <v>-0.6967530397559152</v>
+        <v>-0.05833909940710091</v>
       </c>
       <c r="N85" s="3" t="n">
-        <v>134.844</v>
+        <v>75.06800000000001</v>
       </c>
       <c r="O85" s="3" t="n">
-        <v>132.851</v>
+        <v>74.001</v>
       </c>
       <c r="P85" s="4" t="n">
-        <v>1.50017688989923</v>
+        <v>1.441872407129652</v>
       </c>
       <c r="Q85" s="5" t="n">
-        <v>2.196929929655145</v>
+        <v>1.500211506536753</v>
       </c>
       <c r="R85" t="inlineStr">
         <is>
@@ -5982,7 +5988,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>药</t>
+          <t>互金证券</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -5992,46 +5998,46 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>920367</t>
+          <t>300803</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>新赣江</t>
+          <t>指南针</t>
         </is>
       </c>
       <c r="G86" s="3" t="n">
-        <v>19.95</v>
+        <v>48.38</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>23.8</v>
+        <v>55.17</v>
       </c>
       <c r="I86" s="4" t="n">
-        <v>19.2982456140351</v>
+        <v>14.03472509301364</v>
       </c>
       <c r="J86" s="3" t="n">
-        <v>23.94</v>
+        <v>58.05</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>21.502</v>
+        <v>51.812</v>
       </c>
       <c r="L86" s="3" t="n">
-        <v>21.968</v>
+        <v>52.057</v>
       </c>
       <c r="M86" s="4" t="n">
-        <v>-2.12126729788783</v>
+        <v>-0.4706379545498129</v>
       </c>
       <c r="N86" s="3" t="n">
-        <v>22.098</v>
+        <v>52.79600000000001</v>
       </c>
       <c r="O86" s="3" t="n">
-        <v>21.968</v>
+        <v>52.258</v>
       </c>
       <c r="P86" s="4" t="n">
-        <v>0.5917698470502719</v>
+        <v>1.029507443836364</v>
       </c>
       <c r="Q86" s="5" t="n">
-        <v>2.713037144938102</v>
+        <v>1.500145398386177</v>
       </c>
       <c r="R86" t="inlineStr">
         <is>
@@ -6047,7 +6053,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>药</t>
+          <t>互金证券</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -6057,46 +6063,46 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>688293</t>
+          <t>300085</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>XD奥浦迈</t>
+          <t>银之杰</t>
         </is>
       </c>
       <c r="G87" s="3" t="n">
-        <v>54.08</v>
+        <v>24.89</v>
       </c>
       <c r="H87" s="3" t="n">
-        <v>64.65000000000001</v>
+        <v>28.83</v>
       </c>
       <c r="I87" s="4" t="n">
-        <v>19.54511834319528</v>
+        <v>15.82965046203293</v>
       </c>
       <c r="J87" s="3" t="n">
-        <v>64.89</v>
+        <v>29.86</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>58.05799999999999</v>
+        <v>26.71</v>
       </c>
       <c r="L87" s="3" t="n">
-        <v>59.423</v>
+        <v>26.998</v>
       </c>
       <c r="M87" s="4" t="n">
-        <v>-2.297090352220532</v>
+        <v>-1.066745684865533</v>
       </c>
       <c r="N87" s="3" t="n">
-        <v>59.706</v>
+        <v>27.322</v>
       </c>
       <c r="O87" s="3" t="n">
-        <v>59.70399999999999</v>
+        <v>27.123</v>
       </c>
       <c r="P87" s="4" t="n">
-        <v>0.003349859305923353</v>
+        <v>0.7336946502968011</v>
       </c>
       <c r="Q87" s="5" t="n">
-        <v>2.300440211526456</v>
+        <v>1.800440335162334</v>
       </c>
       <c r="R87" t="inlineStr">
         <is>
@@ -6112,7 +6118,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>电网设备</t>
+          <t>黄金白银</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -6122,46 +6128,46 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>300069</t>
+          <t>300945</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>金利华电</t>
+          <t>曼卡龙</t>
         </is>
       </c>
       <c r="G88" s="3" t="n">
-        <v>21.06</v>
+        <v>10.02</v>
       </c>
       <c r="H88" s="3" t="n">
-        <v>23.99</v>
+        <v>11.52</v>
       </c>
       <c r="I88" s="4" t="n">
-        <v>13.91263057929724</v>
+        <v>14.97005988023952</v>
       </c>
       <c r="J88" s="3" t="n">
-        <v>25.27</v>
+        <v>12.02</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>21.766</v>
+        <v>10.506</v>
       </c>
       <c r="L88" s="3" t="n">
-        <v>22.147</v>
+        <v>10.536</v>
       </c>
       <c r="M88" s="4" t="n">
-        <v>-1.720323294351378</v>
+        <v>-0.2847380410022526</v>
       </c>
       <c r="N88" s="3" t="n">
-        <v>22.318</v>
+        <v>10.762</v>
       </c>
       <c r="O88" s="3" t="n">
-        <v>22.316</v>
+        <v>10.632</v>
       </c>
       <c r="P88" s="4" t="n">
-        <v>0.008962179602090004</v>
+        <v>1.222723852520691</v>
       </c>
       <c r="Q88" s="5" t="n">
-        <v>1.729285473953468</v>
+        <v>1.507461893522943</v>
       </c>
       <c r="R88" t="inlineStr">
         <is>
@@ -6187,46 +6193,46 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>301082</t>
+          <t>300069</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>久盛电气</t>
+          <t>金利华电</t>
         </is>
       </c>
       <c r="G89" s="3" t="n">
-        <v>8.779999999999999</v>
+        <v>21.06</v>
       </c>
       <c r="H89" s="3" t="n">
-        <v>10.23</v>
+        <v>23.99</v>
       </c>
       <c r="I89" s="4" t="n">
-        <v>16.51480637813214</v>
+        <v>13.91263057929724</v>
       </c>
       <c r="J89" s="3" t="n">
-        <v>10.53</v>
+        <v>25.27</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>9.296000000000001</v>
+        <v>21.766</v>
       </c>
       <c r="L89" s="3" t="n">
-        <v>9.324000000000002</v>
+        <v>22.147</v>
       </c>
       <c r="M89" s="4" t="n">
-        <v>-0.3003003003003046</v>
+        <v>-1.720323294351378</v>
       </c>
       <c r="N89" s="3" t="n">
-        <v>9.526</v>
+        <v>22.318</v>
       </c>
       <c r="O89" s="3" t="n">
-        <v>9.413</v>
+        <v>22.316</v>
       </c>
       <c r="P89" s="4" t="n">
-        <v>1.200467438648678</v>
+        <v>0.008962179602090004</v>
       </c>
       <c r="Q89" s="5" t="n">
-        <v>1.500767738948983</v>
+        <v>1.729285473953468</v>
       </c>
       <c r="R89" t="inlineStr">
         <is>
@@ -6252,55 +6258,185 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
+          <t>301082</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>久盛电气</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="n">
+        <v>8.779999999999999</v>
+      </c>
+      <c r="H90" s="3" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="I90" s="4" t="n">
+        <v>16.51480637813214</v>
+      </c>
+      <c r="J90" s="3" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="K90" s="3" t="n">
+        <v>9.296000000000001</v>
+      </c>
+      <c r="L90" s="3" t="n">
+        <v>9.324000000000002</v>
+      </c>
+      <c r="M90" s="4" t="n">
+        <v>-0.3003003003003046</v>
+      </c>
+      <c r="N90" s="3" t="n">
+        <v>9.526</v>
+      </c>
+      <c r="O90" s="3" t="n">
+        <v>9.413</v>
+      </c>
+      <c r="P90" s="4" t="n">
+        <v>1.200467438648678</v>
+      </c>
+      <c r="Q90" s="5" t="n">
+        <v>1.500767738948983</v>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>涨停内可达</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>电网设备</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>空</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
           <t>300427</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr">
+      <c r="F91" t="inlineStr">
         <is>
           <t>红相股份</t>
         </is>
       </c>
-      <c r="G90" s="3" t="n">
+      <c r="G91" s="3" t="n">
         <v>5.21</v>
       </c>
-      <c r="H90" s="3" t="n">
+      <c r="H91" s="3" t="n">
         <v>6.14</v>
       </c>
-      <c r="I90" s="4" t="n">
+      <c r="I91" s="4" t="n">
         <v>17.85028790786946</v>
       </c>
-      <c r="J90" s="3" t="n">
+      <c r="J91" s="3" t="n">
         <v>6.25</v>
       </c>
-      <c r="K90" s="3" t="n">
+      <c r="K91" s="3" t="n">
         <v>5.538</v>
       </c>
-      <c r="L90" s="3" t="n">
+      <c r="L91" s="3" t="n">
         <v>5.588</v>
       </c>
-      <c r="M90" s="4" t="n">
+      <c r="M91" s="4" t="n">
         <v>-0.8947745168217613</v>
       </c>
-      <c r="N90" s="3" t="n">
+      <c r="N91" s="3" t="n">
         <v>5.678</v>
       </c>
-      <c r="O90" s="3" t="n">
+      <c r="O91" s="3" t="n">
         <v>5.643000000000001</v>
       </c>
-      <c r="P90" s="4" t="n">
+      <c r="P91" s="4" t="n">
         <v>0.6202374623427209</v>
       </c>
-      <c r="Q90" s="5" t="n">
+      <c r="Q91" s="5" t="n">
         <v>1.515011979164482</v>
       </c>
-      <c r="R90" t="inlineStr">
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>涨停内可达</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>商业航天</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>空</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>688323</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>瑞华泰</t>
+        </is>
+      </c>
+      <c r="G92" s="3" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="H92" s="3" t="n">
+        <v>21.78</v>
+      </c>
+      <c r="I92" s="4" t="n">
+        <v>19.01639344262296</v>
+      </c>
+      <c r="J92" s="3" t="n">
+        <v>21.96</v>
+      </c>
+      <c r="K92" s="3" t="n">
+        <v>19.84</v>
+      </c>
+      <c r="L92" s="3" t="n">
+        <v>19.986</v>
+      </c>
+      <c r="M92" s="4" t="n">
+        <v>-0.7305113579505473</v>
+      </c>
+      <c r="N92" s="3" t="n">
+        <v>20.312</v>
+      </c>
+      <c r="O92" s="3" t="n">
+        <v>20.156</v>
+      </c>
+      <c r="P92" s="4" t="n">
+        <v>0.7739630879142867</v>
+      </c>
+      <c r="Q92" s="5" t="n">
+        <v>1.504474445864834</v>
+      </c>
+      <c r="R92" t="inlineStr">
         <is>
           <t>涨停内可达</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:R90"/>
+  <autoFilter ref="A2:R92"/>
   <mergeCells count="1">
     <mergeCell ref="A1:R1"/>
   </mergeCells>

</xml_diff>